<commit_message>
Rangement : TODO reecrit, outils remplaces marques, taches completees
TODO.md etait en desordre : sur 25 taches en attente, une douzaine etaient
deja faites. Reecrit et reorganise par destinataire, avec un journal des
travaux acheves par date.

MES_TACHES.xlsx complete de trois taches oubliees : contacter Paye Ton
Influence, demander a L214 et Foodwatch si le registre existe deja, et
solliciter l ARPP. Les deux premieres etaient inscrites depuis la premiere
session et n avaient jamais ete transmises a Vincent.

Deux outils remplaces par surveiller_youtube.py portent desormais un en-tete
qui le dit. Ils sont conserves : des mesures enregistrees ont ete produites
par eux, les supprimer les rendrait irreproductibles.

A_COMPLETER.xlsx recoit un onglet ACHEVE. LISEZ-MOI liste les quinze outils
courants et distingue les classeurs actifs des classeurs acheves.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DfPtphAAkK24cZ5SByH1EW
</commit_message>
<xml_diff>
--- a/cartographie/MES_TACHES.xlsx
+++ b/cartographie/MES_TACHES.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. ALIAS A CHERCHER" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1. MES TACHES'!$A$1:$G$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1. MES TACHES'!$A$1:$G$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2. COMPTES A RELEVER'!$A$1:$H$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3. ALIAS A CHERCHER'!$A$1:$F$9</definedName>
   </definedNames>
@@ -706,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1004,31 +1004,112 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Decider : qui publie le registre ?</t>
+          <t>Contacter Paye Ton Influence</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Toi en nom propre, une association existante, une nouvelle structure ? Question ouverte depuis la premiere session.</t>
+          <t>Pas pour leurs donnees — ils n'en ont pas d'exportables — mais comme partenaire de diffusion. Ils travaillent deja Interbev et Cniel.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>reflexion</t>
+          <t>~20 min</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Determine la posture juridique. Bloque toute publication.</t>
+          <t>Partenaire naturel. Et ils sauront peut-etre si quelqu'un tient deja un registre de ce type, ce qui eviterait de refaire un travail existant.</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr"/>
       <c r="G11" s="6" t="inlineStr"/>
     </row>
+    <row r="12" ht="96" customHeight="1">
+      <c r="A12" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Demander a L214 et Foodwatch si le registre existe deja</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Un message a chacune. Question simple : quelqu'un tient-il deja une base des collaborations entre createurs et industrie animale ?</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>~20 min</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Si oui, on collabore au lieu de dupliquer. Si non, c'est une confirmation que le creneau est libre. Inscrit depuis la premiere session, jamais fait.</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr"/>
+      <c r="G12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13" ht="96" customHeight="1">
+      <c r="A13" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Demander a l'ARPP les donnees brutes de son Observatoire</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>L'Autorite de Regulation Professionnelle de la Publicite analyse de gros volumes (13 356 contenus au 1er semestre 2024) mais ne publie que des agregats.</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>~15 min</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Un refus est lui-meme documentable et cite-able. Le cout est nul, le gain potentiel eleve. METHODOLOGIE section 5.</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr"/>
+      <c r="G13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14" ht="96" customHeight="1">
+      <c r="A14" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Decider : qui publie le registre ?</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Toi en nom propre, une association existante, une nouvelle structure ? Question ouverte depuis la premiere session.</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>reflexion</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Determine la posture juridique. Bloque toute publication.</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr"/>
+      <c r="G14" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G11"/>
+  <autoFilter ref="A1:G14"/>
   <dataValidations count="1">
-    <dataValidation sqref="F2 F3 F4 F5 F6 F7 F8 F9 F10 F11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2 F3 F4 F5 F6 F7 F8 F9 F10 F11 F12 F13 F14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"fait,en cours,pas encore,bloque"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>